<commit_message>
Adiciona o cenário 8 (falha do tratamento químico) e atualiza o estado do projeto
Cenário 8: procedimento por fases e ramos (subdosagem, sobredosagem ou
produto errado, derrame, torre parada ou seca, causa indefinida), com
segurança química em primeiro lugar (FISPQ, não misturar produtos, a
ronda contém, avisa e aciona), parada controlada da torre ou do chiller
e remissão ao cenário 1 se produto ou corante aparecer na torneira.
Fluxograma de 1 página A3/A4, PDF e Word.

Atualiza LEIAME das entregas, o texto da planilha-mestre, a spec
(checklists de rotina feitos; cenários 2, 3, 5, 8, 9 feitos) e o MEMORY.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015N8NW4o2BbADwSCH4ZsDyY
</commit_message>
<xml_diff>
--- a/entregas/plano-contingencia-agua/planilha-mestre/planilha-mestre.xlsx
+++ b/entregas/plano-contingencia-agua/planilha-mestre/planilha-mestre.xlsx
@@ -716,7 +716,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="60" customHeight="1">
+    <row r="9" ht="75" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Cenários</t>
@@ -724,7 +724,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>1 Contaminação cruzada · 2 Falta de água · 3 Água fora do padrão · 4 Vazamento e alagamento · 5 Falha de bomba ou energia · 6 Incêndio com reserva indisponível · 7 Refluxo de esgoto · 8 Falha do tratamento químico · 9 Contaminação do reservatório · T Comunicação de crise. Os procedimentos dos cenários 1, 2 e 5 estão em entregas/plano-contingencia-agua/cenarios/.</t>
+          <t>1 Contaminação cruzada · 2 Falta de água · 3 Água fora do padrão · 4 Vazamento e alagamento · 5 Falha de bomba ou energia · 6 Incêndio com reserva indisponível · 7 Refluxo de esgoto · 8 Falha do tratamento químico · 9 Contaminação do reservatório · T Comunicação de crise. Os procedimentos dos cenários 1, 2, 3, 5, 8 e 9 estão em entregas/plano-contingencia-agua/cenarios/; os checklists de ronda e do relatório mensal dos fornecedores estão em .../rotinas/.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza pacote de revisão com os cenários 4, 6 e 7 e fecha o estado do projeto
Pacote de revisão: 20 itens de risco (R-15 a R-20 novos: isolar setor de
incêndio para estancar alagamento, gases de esgoto, restringir uso de
água a montante, desenergizar sem habilitado, higienização e descarte,
rede de incêndio), 20 valores a fixar (V-16 a V-20) e 14 decisões de
política (Q-11 a Q-14). Registra que os cenários 4, 6 e 7 ainda não
foram conferidos contra os demais e que só falta o cenário T.

LEIAME, texto da planilha-mestre, spec e MEMORY atualizados.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015N8NW4o2BbADwSCH4ZsDyY
</commit_message>
<xml_diff>
--- a/entregas/plano-contingencia-agua/planilha-mestre/planilha-mestre.xlsx
+++ b/entregas/plano-contingencia-agua/planilha-mestre/planilha-mestre.xlsx
@@ -716,7 +716,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="75" customHeight="1">
+    <row r="9" ht="90" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Cenários</t>
@@ -724,7 +724,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>1 Contaminação cruzada · 2 Falta de água · 3 Água fora do padrão · 4 Vazamento e alagamento · 5 Falha de bomba ou energia · 6 Incêndio com reserva indisponível · 7 Refluxo de esgoto · 8 Falha do tratamento químico · 9 Contaminação do reservatório · T Comunicação de crise. Os procedimentos dos cenários 1, 2, 3, 5, 8 e 9 estão em entregas/plano-contingencia-agua/cenarios/; os checklists de ronda e do relatório mensal dos fornecedores estão em .../rotinas/.</t>
+          <t>1 Contaminação cruzada · 2 Falta de água · 3 Água fora do padrão · 4 Vazamento e alagamento · 5 Falha de bomba ou energia · 6 Incêndio com reserva indisponível · 7 Refluxo de esgoto · 8 Falha do tratamento químico · 9 Contaminação do reservatório · T Comunicação de crise. Os procedimentos dos cenários 1 a 9 (o T, comunicação de crise, ainda não existe) estão em entregas/plano-contingencia-agua/cenarios/; os checklists de ronda e do relatório mensal dos fornecedores estão em .../rotinas/.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Uniformiza os cenários e aplica página nova por seção longa
Passada de consistência entre os cenários 1 a 9: remoção do número de
telefone do centro toxicológico (não confirmado), monitoramento reforçado
como sugestão de 30 dias a validar pelo responsável técnico, ponteiro
para o Cenário T (graus G1/G2/G3 e modelos-padrão) em todos os cenários.
Pacote de revisão e planilha ajustados. Todos os PDF, Word e fluxogramas
regerados; seções longas começam em página nova, como nos modelos DF.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015N8NW4o2BbADwSCH4ZsDyY
</commit_message>
<xml_diff>
--- a/entregas/plano-contingencia-agua/planilha-mestre/planilha-mestre.xlsx
+++ b/entregas/plano-contingencia-agua/planilha-mestre/planilha-mestre.xlsx
@@ -1873,7 +1873,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Disque-Intoxicação (confirmar número vigente)</t>
+          <t>Centro de informação toxicológica (telefone a confirmar)</t>
         </is>
       </c>
       <c r="B18" s="17" t="inlineStr">
@@ -1886,7 +1886,7 @@
       <c r="E18" s="14" t="n"/>
       <c r="F18" s="14" t="inlineStr">
         <is>
-          <t>Anvisa: 0800 722 6001 — conferir se continua vigente antes de usar</t>
+          <t>Preencher com o telefone do centro de informação toxicológica (confirmar o número vigente)</t>
         </is>
       </c>
     </row>

</xml_diff>